<commit_message>
ajustement de la partie resultat
</commit_message>
<xml_diff>
--- a/public/modele_creation.xlsx
+++ b/public/modele_creation.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
   <si>
     <t>Key</t>
   </si>
@@ -30,10 +30,7 @@
     <t/>
   </si>
   <si>
-    <t>Entreprise</t>
-  </si>
-  <si>
-    <t>Numero_Enregistrement</t>
+    <t>Organisation</t>
   </si>
   <si>
     <t>Secteur</t>
@@ -524,7 +521,7 @@
   <sheetPr>
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15.6" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.09765625" style="1" customWidth="1"/>
@@ -600,7 +597,7 @@
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>3</v>
       </c>
     </row>
@@ -616,15 +613,7 @@
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -650,39 +639,39 @@
         <v>2</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -700,31 +689,31 @@
   <sheetData>
     <row r="1" ht="16.2" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>